<commit_message>
refactor: Update ISEC calculation with a pair-specific frequency numerator and explicit alpha weighting, increase top K matches, and adjust data file paths.
</commit_message>
<xml_diff>
--- a/ISEC_Results.xlsx
+++ b/ISEC_Results.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -488,7 +488,7 @@
         <v>100</v>
       </c>
       <c r="D2" t="n">
-        <v>1.1772</v>
+        <v>3</v>
       </c>
       <c r="E2" t="n">
         <v>1</v>
@@ -513,13 +513,13 @@
         <v>3.3289</v>
       </c>
       <c r="K2" t="n">
-        <v>0.4396</v>
+        <v>5.7489</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Limpia tapicería y alfombras Binner</t>
+          <t>Limpia tapicería en espuma Binner</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -528,17 +528,17 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Limpia tapicería en espuma Binner</t>
+          <t>Limpiador Dr. Beckmann alfombras 2 en 1 poder oxi x 650 ml</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -547,22 +547,22 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="I3" t="n">
-        <v>0.0751</v>
+        <v>0.256</v>
       </c>
       <c r="J3" t="n">
-        <v>3.3289</v>
+        <v>11.2248</v>
       </c>
       <c r="K3" t="n">
-        <v>0.3734</v>
+        <v>1.6167</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Limpiador Dr. Beckmann alfombras 2 en 1 poder oxi x 650 ml</t>
+          <t>Limpia tapicería y alfombras Binner</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -571,35 +571,164 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="D4" t="n">
-        <v>0.5886</v>
+        <v>2.699</v>
       </c>
       <c r="E4" t="n">
         <v>1</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
+          <t>Limpia tapicería en espuma Binner</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>100</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.0751</v>
+      </c>
+      <c r="J4" t="n">
+        <v>3.3289</v>
+      </c>
+      <c r="K4" t="n">
+        <v>5.7489</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
           <t>Limpia tapicería y alfombras Binner</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H4" t="n">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
         <v>50</v>
       </c>
-      <c r="I4" t="n">
+      <c r="D5" t="n">
+        <v>2.699</v>
+      </c>
+      <c r="E5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Limpiador Dr. Beckmann alfombras 2 en 1 poder oxi x 650 ml</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>10</v>
+      </c>
+      <c r="I5" t="n">
         <v>0.2454</v>
       </c>
-      <c r="J4" t="n">
+      <c r="J5" t="n">
         <v>9.6143</v>
       </c>
-      <c r="K4" t="n">
-        <v>0.076</v>
+      <c r="K5" t="n">
+        <v>1.6127</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Limpiador Dr. Beckmann alfombras 2 en 1 poder oxi x 650 ml</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>10</v>
+      </c>
+      <c r="D6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Limpia tapicería y alfombras Binner</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>50</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.2454</v>
+      </c>
+      <c r="J6" t="n">
+        <v>9.6143</v>
+      </c>
+      <c r="K6" t="n">
+        <v>1.6127</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Limpiador Dr. Beckmann alfombras 2 en 1 poder oxi x 650 ml</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>10</v>
+      </c>
+      <c r="D7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Limpia tapicería en espuma Binner</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>100</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.256</v>
+      </c>
+      <c r="J7" t="n">
+        <v>11.2248</v>
+      </c>
+      <c r="K7" t="n">
+        <v>1.6167</v>
       </c>
     </row>
   </sheetData>

</xml_diff>